<commit_message>
Worked on PCB BOM
</commit_message>
<xml_diff>
--- a/hardware/pcb/Smart Switch BOM.xlsx
+++ b/hardware/pcb/Smart Switch BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Code\ICAMS\zigbee-smart-switch\hardware\pcb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F03057-5F9A-499F-AD0E-B1A92825ABA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29967E3-1827-4E8C-BEA0-8AE2DB9F73F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="101">
   <si>
     <t>Coordinator</t>
   </si>
@@ -249,15 +249,6 @@
     <t>Connects line in and line out</t>
   </si>
   <si>
-    <t>Male Wall Blades</t>
-  </si>
-  <si>
-    <t>Female Wall Blades</t>
-  </si>
-  <si>
-    <t>12 AWG Wire</t>
-  </si>
-  <si>
     <t>Main in source</t>
   </si>
   <si>
@@ -265,6 +256,78 @@
   </si>
   <si>
     <t>Main connections</t>
+  </si>
+  <si>
+    <t>U.FL to RP-SMA</t>
+  </si>
+  <si>
+    <t>Male Plug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4GHZ DIPOLE ANTENNA RP-SMA </t>
+  </si>
+  <si>
+    <t>Antenna for range</t>
+  </si>
+  <si>
+    <t>Connects antenna to XBee3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 AWG Wire 10' </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female Plug </t>
+  </si>
+  <si>
+    <t>$3.76 (each)</t>
+  </si>
+  <si>
+    <t>$3.98 (each)</t>
+  </si>
+  <si>
+    <t>$6.97 (each)</t>
+  </si>
+  <si>
+    <t>$16.79 (each, 10')</t>
+  </si>
+  <si>
+    <t>$2.94 (each)</t>
+  </si>
+  <si>
+    <t>PCB Manufacturers:</t>
+  </si>
+  <si>
+    <t>Manufacturuer</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Lead time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB Way </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green Circuits </t>
+  </si>
+  <si>
+    <t>EMSG</t>
+  </si>
+  <si>
+    <t>AlteraFlex</t>
+  </si>
+  <si>
+    <t>PCC</t>
+  </si>
+  <si>
+    <t>Coordinator size:</t>
+  </si>
+  <si>
+    <t>Joiner Control size:</t>
+  </si>
+  <si>
+    <t>Joiner Power Size:</t>
   </si>
 </sst>
 </file>
@@ -291,15 +354,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -307,27 +382,157 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -609,545 +814,686 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" customWidth="1"/>
     <col min="2" max="2" width="7.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
     <col min="4" max="4" width="33.5703125" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="10.5703125" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="H1" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="23" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="H2" s="28"/>
+      <c r="I2" s="29" t="s">
+        <v>0</v>
+      </c>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="F3" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="J3" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="K3" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="N3" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="O3" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="P3" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q3" s="30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="5">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="25" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="H4" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="8">
         <v>20.36</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="F5" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="5">
         <v>1</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="10">
         <v>2.95</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F6" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="24" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="H7" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="5">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="26" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="H8" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="4">
         <v>1</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="5">
         <v>2</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="26" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="4">
         <v>2</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="5">
         <v>1</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="10">
         <v>0.14000000000000001</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="F12" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="4">
         <v>22</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="F13" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="5">
         <v>22</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="F14" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="6">
         <v>3</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="F15" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="5">
         <v>2</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="10">
         <v>0.42</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="F16" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="4">
         <v>22</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="F17" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="5">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="F18" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="4">
         <v>10</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="F19" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="5">
         <v>10</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="F20" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="4">
         <v>10</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="F21" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="5">
         <v>10</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="F22" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="4">
         <v>10</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="F23" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="5">
         <v>10</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="F24" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="4">
         <v>20</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="F25" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B26" s="5">
+        <v>10</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="4">
+        <v>10</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F27" s="24" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="5">
+        <v>2</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>75</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="B29" s="4">
+        <v>10</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E28" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>8</v>
+      <c r="B30" s="7">
+        <v>10</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="H30" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="O2:Q2"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" xr:uid="{7AF628B5-7A69-4E2D-9995-33C855D081C2}"/>
     <hyperlink ref="A4" r:id="rId2" xr:uid="{D974D2AE-2329-4226-9DC1-754731DED559}"/>
@@ -1167,8 +1513,18 @@
     <hyperlink ref="A24" r:id="rId16" xr:uid="{56599617-85B3-436F-9232-3D0E1F35E3B7}"/>
     <hyperlink ref="A23" r:id="rId17" xr:uid="{4823A820-C64D-4BAB-AAD8-C4658B1D84A2}"/>
     <hyperlink ref="A25" r:id="rId18" xr:uid="{7931AF2F-09A7-42C9-AE3D-275FFDC8E27C}"/>
+    <hyperlink ref="A30" r:id="rId19" xr:uid="{32C5FDA1-1E59-47E9-AC86-F5B0AC89972A}"/>
+    <hyperlink ref="A29" r:id="rId20" xr:uid="{1BBE7309-D7C7-4575-930D-DD93C0AA3635}"/>
+    <hyperlink ref="A28" r:id="rId21" xr:uid="{A1AAAABE-1E43-4443-B825-943B5D59970F}"/>
+    <hyperlink ref="A27" r:id="rId22" xr:uid="{CF64D41B-8B05-481F-96A7-68DB6E956FC4}"/>
+    <hyperlink ref="A26" r:id="rId23" xr:uid="{44D6262B-B52A-4692-AF73-869809C86489}"/>
+    <hyperlink ref="H4" r:id="rId24" xr:uid="{90283C41-A4CE-473A-8CB6-A769C4A2D877}"/>
+    <hyperlink ref="H5" r:id="rId25" xr:uid="{F3A6CF93-8AC1-44AB-8437-8A07B84FA4B5}"/>
+    <hyperlink ref="H6" r:id="rId26" xr:uid="{B8C6D6A4-3FE9-44EB-B5ED-C2C39EC96876}"/>
+    <hyperlink ref="H7" r:id="rId27" xr:uid="{FF1864B5-5D0A-4AE7-A517-D32D8836D970}"/>
+    <hyperlink ref="H8" r:id="rId28" xr:uid="{E021E953-3AE4-4EB0-B8E5-8BE13381304D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId19"/>
+  <pageSetup orientation="portrait" r:id="rId29"/>
 </worksheet>
 </file>
</xml_diff>